<commit_message>
update data package at: 2026-09-25T11:52:10
</commit_message>
<xml_diff>
--- a/data/BASE_INTRA_ORCAMENTARIA_REPASSE.xlsx
+++ b/data/BASE_INTRA_ORCAMENTARIA_REPASSE.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 5</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 24</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 4</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>3 3 91 39</t>
+          <t>3 3 91 39 20</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -4871,7 +4871,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -4912,7 +4912,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -5568,7 +5568,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -5650,7 +5650,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>3 1 91 04</t>
+          <t>3 1 91 4 4</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 24</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -5773,7 +5773,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 24</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -6101,7 +6101,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 24</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 24</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -6716,7 +6716,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -6757,7 +6757,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -7003,7 +7003,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -7085,7 +7085,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -7126,7 +7126,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -7249,7 +7249,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -7331,7 +7331,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 24</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -7413,7 +7413,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -7454,7 +7454,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -7495,7 +7495,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -7700,7 +7700,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -7741,7 +7741,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>3 3 91 39</t>
+          <t>3 3 91 39 20</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>3 3 91 39</t>
+          <t>3 3 91 39 20</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -7905,7 +7905,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>4 6 91 93</t>
+          <t>4 6 91 93 31</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -7946,7 +7946,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>3 3 91 30</t>
+          <t>3 3 91 30 8</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>3 3 91 30</t>
+          <t>3 3 91 30 8</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -8028,7 +8028,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>3 3 91 30</t>
+          <t>3 3 91 30 8</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>3 3 91 30</t>
+          <t>3 3 91 30 8</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>3 3 91 30</t>
+          <t>3 3 91 30 8</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -8151,7 +8151,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -8192,7 +8192,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -8397,7 +8397,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -8520,7 +8520,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -8684,7 +8684,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -8725,7 +8725,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -8766,7 +8766,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
@@ -8807,7 +8807,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 8</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -8889,7 +8889,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
@@ -8930,7 +8930,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>3 2 91 21</t>
+          <t>3 2 91 21 3</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>4 6 91 71</t>
+          <t>4 6 91 71 3</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>3 3 91 40</t>
+          <t>3 3 91 40 2</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
@@ -9053,7 +9053,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>3 3 91 39</t>
+          <t>3 3 91 39 28</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
@@ -9135,7 +9135,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -9217,7 +9217,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
@@ -9258,7 +9258,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>3 3 91 39</t>
+          <t>3 3 91 39 28</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>3 3 91 39</t>
+          <t>3 3 91 39 29</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
@@ -9340,7 +9340,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>3 3 91 39</t>
+          <t>3 3 91 39 98</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
@@ -9381,7 +9381,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -9422,7 +9422,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>4 5 91 41</t>
+          <t>4 5 91 41 3</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -9463,7 +9463,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -9504,7 +9504,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
@@ -9545,7 +9545,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -9586,7 +9586,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
@@ -9627,7 +9627,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>3 3 91 41</t>
+          <t>3 3 91 41 4</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
@@ -9709,7 +9709,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -9750,7 +9750,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -9791,7 +9791,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -9832,7 +9832,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>3 1 91 92</t>
+          <t>3 1 91 92 3</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>3 1 91 92</t>
+          <t>3 1 91 92 3</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
@@ -9996,7 +9996,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -10037,7 +10037,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -10078,7 +10078,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -10160,7 +10160,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
@@ -10201,7 +10201,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -10242,7 +10242,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -10283,7 +10283,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -10324,7 +10324,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -10365,7 +10365,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -10447,7 +10447,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -10529,7 +10529,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -10652,7 +10652,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -10693,7 +10693,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -10857,7 +10857,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -10898,7 +10898,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -10980,7 +10980,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -11021,7 +11021,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -11062,7 +11062,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -11144,7 +11144,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -11185,7 +11185,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -11267,7 +11267,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -11390,7 +11390,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -11431,7 +11431,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -11513,7 +11513,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -11595,7 +11595,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
@@ -11636,7 +11636,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -11677,7 +11677,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -11759,7 +11759,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -11800,7 +11800,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -11841,7 +11841,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -11882,7 +11882,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -11964,7 +11964,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -12046,7 +12046,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -12087,7 +12087,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -12169,7 +12169,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -12210,7 +12210,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -12251,7 +12251,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -12292,7 +12292,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -12415,7 +12415,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -12497,7 +12497,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -12538,7 +12538,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -12620,7 +12620,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -12743,7 +12743,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -12784,7 +12784,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -12825,7 +12825,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -12866,7 +12866,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
@@ -12948,7 +12948,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -12989,7 +12989,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
@@ -13030,7 +13030,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -13071,7 +13071,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -13112,7 +13112,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -13153,7 +13153,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -13194,7 +13194,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
@@ -13235,7 +13235,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -13317,7 +13317,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -13358,7 +13358,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -13399,7 +13399,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -13440,7 +13440,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -13481,7 +13481,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -13522,7 +13522,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -13563,7 +13563,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
@@ -13604,7 +13604,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -13645,7 +13645,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -13727,7 +13727,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
@@ -13768,7 +13768,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
@@ -13809,7 +13809,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
@@ -13850,7 +13850,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
@@ -13891,7 +13891,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
@@ -13932,7 +13932,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
@@ -14014,7 +14014,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
@@ -14055,7 +14055,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
@@ -14137,7 +14137,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
@@ -14178,7 +14178,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
@@ -14219,7 +14219,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
@@ -14260,7 +14260,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
@@ -14301,7 +14301,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
@@ -14383,7 +14383,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
@@ -14424,7 +14424,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
@@ -14465,7 +14465,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
@@ -14506,7 +14506,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
@@ -14547,7 +14547,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
@@ -14629,7 +14629,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
@@ -14670,7 +14670,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
@@ -14711,7 +14711,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
@@ -14752,7 +14752,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
@@ -14793,7 +14793,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
@@ -14834,7 +14834,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
@@ -14875,7 +14875,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
@@ -14916,7 +14916,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -14957,7 +14957,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
@@ -14998,7 +14998,7 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
@@ -15039,7 +15039,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -15080,7 +15080,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
@@ -15121,7 +15121,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
@@ -15162,7 +15162,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
@@ -15244,7 +15244,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
@@ -15326,7 +15326,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
@@ -15367,7 +15367,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
@@ -15408,7 +15408,7 @@
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
@@ -15449,7 +15449,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
@@ -15490,7 +15490,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
@@ -15531,7 +15531,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
@@ -15572,7 +15572,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
@@ -15613,7 +15613,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
@@ -15695,7 +15695,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
@@ -15777,7 +15777,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
@@ -15818,7 +15818,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 26</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
@@ -15859,7 +15859,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 8</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
@@ -15941,7 +15941,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
@@ -15982,7 +15982,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
@@ -16023,7 +16023,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
@@ -16064,7 +16064,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 5</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 21</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
@@ -16146,7 +16146,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 6</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
@@ -16187,7 +16187,7 @@
       </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 22</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
@@ -16228,7 +16228,7 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>3 1 91 13</t>
+          <t>3 1 91 13 8</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">

</xml_diff>